<commit_message>
Big update, haven't updated in a long time, various changes, lap sections by both BR2 and mylaps, liftAndCoast logic
</commit_message>
<xml_diff>
--- a/trackDB/seasonOverview.xlsx
+++ b/trackDB/seasonOverview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SimEnv\trackDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25F67609-F366-410B-B618-845ACB414EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FF6518-034E-4F85-A2BC-699888C81108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39255" yWindow="2490" windowWidth="18180" windowHeight="13740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Track</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>AGP</t>
+  </si>
+  <si>
+    <t>TAU</t>
+  </si>
+  <si>
+    <t>RUA</t>
+  </si>
+  <si>
+    <t>TAS</t>
   </si>
 </sst>
 </file>
@@ -363,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -417,6 +426,57 @@
         <v>290</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>84</v>
+      </c>
+      <c r="C4">
+        <v>200</v>
+      </c>
+      <c r="D4">
+        <v>200</v>
+      </c>
+      <c r="E4">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>75</v>
+      </c>
+      <c r="C5">
+        <v>200</v>
+      </c>
+      <c r="D5">
+        <v>200</v>
+      </c>
+      <c r="E5">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>40</v>
+      </c>
+      <c r="C6">
+        <v>280</v>
+      </c>
+      <c r="D6">
+        <v>200</v>
+      </c>
+      <c r="E6">
+        <v>280</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>